<commit_message>
changed source plates and added new experiment scripts
</commit_message>
<xml_diff>
--- a/crisscross_kit/crisscross/dna_source_plates/cargo_plates/P3510_SSW_cnt_patterning.xlsx
+++ b/crisscross_kit/crisscross/dna_source_plates/cargo_plates/P3510_SSW_cnt_patterning.xlsx
@@ -1,22 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stellawang/Documents/gitrepos/Crisscross-Design/crisscross_kit/crisscross/dna_source_plates/cargo_plates/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05911FD-561F-154F-B8CE-FA8DEA67AF1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-10540" yWindow="-25700" windowWidth="47420" windowHeight="21300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Data" sheetId="1" r:id="rId1"/>
     <sheet name="2D Layout" sheetId="2" r:id="rId2"/>
     <sheet name="2D Label" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="750">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1026" uniqueCount="757">
   <si>
     <t>well</t>
   </si>
@@ -2266,13 +2272,34 @@
   </si>
   <si>
     <t>P</t>
+  </si>
+  <si>
+    <t>CATTTTTGCGGAATTCCATATAACAGTTGAATTTGGGGCGCG tt ATAAAAGCAT</t>
+  </si>
+  <si>
+    <t>Cargo Handle For Slat Position 12, Side h2, Cargo ID SW066GoldNanowireAntiHandle10nt, ordered as SSW109</t>
+  </si>
+  <si>
+    <t>CARGO-SW066GoldNanowireAntiHandle10nt-h2-position_12</t>
+  </si>
+  <si>
+    <t>NON-SLAT OLIGO</t>
+  </si>
+  <si>
+    <t>TTTTTTTTTT</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Obsolete well, may be contaminated, do not use</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2288,8 +2315,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2305,6 +2338,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0000FF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD3D3D3"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2336,26 +2375,37 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2393,7 +2443,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -2427,6 +2477,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -2461,9 +2512,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2636,18 +2688,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E385"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" customWidth="1"/>
-    <col min="2" max="2" width="54.7109375" customWidth="1"/>
-    <col min="3" max="3" width="69.7109375" customWidth="1"/>
-    <col min="4" max="4" width="86.7109375" customWidth="1"/>
-    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="6.6640625" customWidth="1"/>
+    <col min="2" max="2" width="54.6640625" customWidth="1"/>
+    <col min="3" max="3" width="69.6640625" customWidth="1"/>
+    <col min="4" max="4" width="86.6640625" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2664,7 +2716,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -2681,7 +2733,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -2698,7 +2750,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -2715,7 +2767,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2732,107 +2784,107 @@
         <v>200</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>29</v>
       </c>
@@ -2849,7 +2901,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -2866,7 +2918,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>31</v>
       </c>
@@ -2883,7 +2935,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -2900,7 +2952,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>33</v>
       </c>
@@ -2917,7 +2969,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>34</v>
       </c>
@@ -2934,7 +2986,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>35</v>
       </c>
@@ -2951,7 +3003,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>36</v>
       </c>
@@ -2968,87 +3020,87 @@
         <v>200</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>53</v>
       </c>
@@ -3065,7 +3117,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>54</v>
       </c>
@@ -3082,7 +3134,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>55</v>
       </c>
@@ -3099,7 +3151,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>56</v>
       </c>
@@ -3116,7 +3168,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>57</v>
       </c>
@@ -3133,7 +3185,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>58</v>
       </c>
@@ -3150,7 +3202,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>59</v>
       </c>
@@ -3167,7 +3219,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>60</v>
       </c>
@@ -3184,87 +3236,87 @@
         <v>200</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>77</v>
       </c>
@@ -3281,7 +3333,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>78</v>
       </c>
@@ -3298,7 +3350,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>79</v>
       </c>
@@ -3315,7 +3367,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>80</v>
       </c>
@@ -3332,7 +3384,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>81</v>
       </c>
@@ -3349,7 +3401,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>82</v>
       </c>
@@ -3366,7 +3418,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>83</v>
       </c>
@@ -3383,7 +3435,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>84</v>
       </c>
@@ -3400,87 +3452,87 @@
         <v>200</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="84" spans="1:5">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="91" spans="1:5">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="96" spans="1:5">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="97" spans="1:5">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="98" spans="1:5">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>101</v>
       </c>
@@ -3497,7 +3549,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="99" spans="1:5">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>102</v>
       </c>
@@ -3514,117 +3566,117 @@
         <v>200</v>
       </c>
     </row>
-    <row r="100" spans="1:5">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="101" spans="1:5">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="108" spans="1:5">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="109" spans="1:5">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="110" spans="1:5">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="111" spans="1:5">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="112" spans="1:5">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="113" spans="1:5">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="114" spans="1:5">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="116" spans="1:5">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="117" spans="1:5">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="118" spans="1:5">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="119" spans="1:5">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="122" spans="1:5">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>125</v>
       </c>
@@ -3641,7 +3693,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="123" spans="1:5">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>126</v>
       </c>
@@ -3658,7 +3710,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="124" spans="1:5">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>127</v>
       </c>
@@ -3675,7 +3727,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="125" spans="1:5">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>128</v>
       </c>
@@ -3692,7 +3744,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="126" spans="1:5">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>129</v>
       </c>
@@ -3709,7 +3761,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="127" spans="1:5">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>130</v>
       </c>
@@ -3726,7 +3778,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="128" spans="1:5">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>131</v>
       </c>
@@ -3743,7 +3795,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="129" spans="1:5">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>132</v>
       </c>
@@ -3760,7 +3812,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="130" spans="1:5">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>133</v>
       </c>
@@ -3777,7 +3829,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="131" spans="1:5">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>134</v>
       </c>
@@ -3794,7 +3846,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="132" spans="1:5">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>135</v>
       </c>
@@ -3811,7 +3863,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="133" spans="1:5">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>136</v>
       </c>
@@ -3828,7 +3880,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="134" spans="1:5">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>137</v>
       </c>
@@ -3845,7 +3897,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="135" spans="1:5">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>138</v>
       </c>
@@ -3862,7 +3914,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="136" spans="1:5">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>139</v>
       </c>
@@ -3879,7 +3931,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="137" spans="1:5">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>140</v>
       </c>
@@ -3896,47 +3948,47 @@
         <v>200</v>
       </c>
     </row>
-    <row r="138" spans="1:5">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="139" spans="1:5">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="140" spans="1:5">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="141" spans="1:5">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="142" spans="1:5">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="143" spans="1:5">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="144" spans="1:5">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="146" spans="1:5">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>149</v>
       </c>
@@ -3953,7 +4005,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="147" spans="1:5">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>150</v>
       </c>
@@ -3970,7 +4022,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="148" spans="1:5">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>151</v>
       </c>
@@ -3987,7 +4039,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="149" spans="1:5">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>152</v>
       </c>
@@ -4004,7 +4056,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="150" spans="1:5">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>153</v>
       </c>
@@ -4021,7 +4073,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="151" spans="1:5">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>154</v>
       </c>
@@ -4038,7 +4090,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="152" spans="1:5">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>155</v>
       </c>
@@ -4055,7 +4107,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="153" spans="1:5">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>156</v>
       </c>
@@ -4072,7 +4124,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="154" spans="1:5">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>157</v>
       </c>
@@ -4089,7 +4141,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="155" spans="1:5">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>158</v>
       </c>
@@ -4106,7 +4158,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="156" spans="1:5">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>159</v>
       </c>
@@ -4123,7 +4175,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="157" spans="1:5">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>160</v>
       </c>
@@ -4140,7 +4192,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="158" spans="1:5">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>161</v>
       </c>
@@ -4157,7 +4209,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="159" spans="1:5">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>162</v>
       </c>
@@ -4174,7 +4226,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="160" spans="1:5">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>163</v>
       </c>
@@ -4191,52 +4243,52 @@
         <v>200</v>
       </c>
     </row>
-    <row r="161" spans="1:5">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="162" spans="1:5">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="163" spans="1:5">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="164" spans="1:5">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="165" spans="1:5">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="166" spans="1:5">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="167" spans="1:5">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="168" spans="1:5">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="169" spans="1:5">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="170" spans="1:5">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>173</v>
       </c>
@@ -4253,7 +4305,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="171" spans="1:5">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>174</v>
       </c>
@@ -4270,7 +4322,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="172" spans="1:5">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>175</v>
       </c>
@@ -4287,7 +4339,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="173" spans="1:5">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>176</v>
       </c>
@@ -4304,107 +4356,107 @@
         <v>200</v>
       </c>
     </row>
-    <row r="174" spans="1:5">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="175" spans="1:5">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="176" spans="1:5">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="177" spans="1:1">
+    <row r="177" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="178" spans="1:1">
+    <row r="178" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="179" spans="1:1">
+    <row r="179" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="180" spans="1:1">
+    <row r="180" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="181" spans="1:1">
+    <row r="181" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="182" spans="1:1">
+    <row r="182" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="183" spans="1:1">
+    <row r="183" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="184" spans="1:1">
+    <row r="184" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="185" spans="1:1">
+    <row r="185" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="186" spans="1:1">
+    <row r="186" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="187" spans="1:1">
+    <row r="187" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="188" spans="1:1">
+    <row r="188" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="189" spans="1:1">
+    <row r="189" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="190" spans="1:1">
+    <row r="190" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="191" spans="1:1">
+    <row r="191" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="192" spans="1:1">
+    <row r="192" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="193" spans="1:5">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="194" spans="1:5">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>197</v>
       </c>
@@ -4421,7 +4473,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="195" spans="1:5">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>198</v>
       </c>
@@ -4438,7 +4490,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="196" spans="1:5">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>199</v>
       </c>
@@ -4455,7 +4507,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="197" spans="1:5">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>200</v>
       </c>
@@ -4472,107 +4524,107 @@
         <v>200</v>
       </c>
     </row>
-    <row r="198" spans="1:5">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="199" spans="1:5">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="200" spans="1:5">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="201" spans="1:5">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="202" spans="1:5">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="203" spans="1:5">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="204" spans="1:5">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="205" spans="1:5">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="206" spans="1:5">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="207" spans="1:5">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="208" spans="1:5">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="209" spans="1:5">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="210" spans="1:5">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="211" spans="1:5">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="212" spans="1:5">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="213" spans="1:5">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="214" spans="1:5">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="215" spans="1:5">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="216" spans="1:5">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="217" spans="1:5">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="218" spans="1:5">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>221</v>
       </c>
@@ -4589,24 +4641,24 @@
         <v>200</v>
       </c>
     </row>
-    <row r="219" spans="1:5">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>222</v>
       </c>
       <c r="B219" t="s">
-        <v>459</v>
+        <v>753</v>
       </c>
       <c r="C219" t="s">
         <v>565</v>
       </c>
       <c r="D219" t="s">
-        <v>673</v>
+        <v>756</v>
       </c>
       <c r="E219">
         <v>200</v>
       </c>
     </row>
-    <row r="220" spans="1:5">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>223</v>
       </c>
@@ -4623,112 +4675,148 @@
         <v>200</v>
       </c>
     </row>
-    <row r="221" spans="1:5">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="222" spans="1:5">
+      <c r="B221" t="s">
+        <v>753</v>
+      </c>
+      <c r="C221" t="s">
+        <v>754</v>
+      </c>
+      <c r="D221" t="s">
+        <v>756</v>
+      </c>
+      <c r="E221">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="223" spans="1:5">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="224" spans="1:5">
+      <c r="B223" t="s">
+        <v>459</v>
+      </c>
+      <c r="C223" t="s">
+        <v>565</v>
+      </c>
+      <c r="D223" t="s">
+        <v>673</v>
+      </c>
+      <c r="E223">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="225" spans="1:1">
+      <c r="B224" t="s">
+        <v>752</v>
+      </c>
+      <c r="C224" s="4" t="s">
+        <v>750</v>
+      </c>
+      <c r="D224" t="s">
+        <v>751</v>
+      </c>
+      <c r="E224">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="226" spans="1:1">
+    <row r="226" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="227" spans="1:1">
+    <row r="227" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="228" spans="1:1">
+    <row r="228" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="229" spans="1:1">
+    <row r="229" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="230" spans="1:1">
+    <row r="230" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="231" spans="1:1">
+    <row r="231" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="232" spans="1:1">
+    <row r="232" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="233" spans="1:1">
+    <row r="233" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="234" spans="1:1">
+    <row r="234" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="235" spans="1:1">
+    <row r="235" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="236" spans="1:1">
+    <row r="236" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="237" spans="1:1">
+    <row r="237" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="238" spans="1:1">
+    <row r="238" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="239" spans="1:1">
+    <row r="239" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="240" spans="1:1">
+    <row r="240" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="241" spans="1:5">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="242" spans="1:5">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>245</v>
       </c>
@@ -4745,7 +4833,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="243" spans="1:5">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>246</v>
       </c>
@@ -4762,7 +4850,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="244" spans="1:5">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>247</v>
       </c>
@@ -4779,7 +4867,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="245" spans="1:5">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>248</v>
       </c>
@@ -4796,107 +4884,107 @@
         <v>200</v>
       </c>
     </row>
-    <row r="246" spans="1:5">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="247" spans="1:5">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="248" spans="1:5">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="249" spans="1:5">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="250" spans="1:5">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="251" spans="1:5">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="252" spans="1:5">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>255</v>
       </c>
     </row>
-    <row r="253" spans="1:5">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="254" spans="1:5">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="255" spans="1:5">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="256" spans="1:5">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="257" spans="1:5">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="258" spans="1:5">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>261</v>
       </c>
     </row>
-    <row r="259" spans="1:5">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="260" spans="1:5">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="261" spans="1:5">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="262" spans="1:5">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="263" spans="1:5">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="264" spans="1:5">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>267</v>
       </c>
     </row>
-    <row r="265" spans="1:5">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="266" spans="1:5">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>269</v>
       </c>
@@ -4913,12 +5001,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="267" spans="1:5">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="268" spans="1:5">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>271</v>
       </c>
@@ -4935,12 +5023,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="269" spans="1:5">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="270" spans="1:5">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>273</v>
       </c>
@@ -4957,12 +5045,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="271" spans="1:5">
+    <row r="271" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="272" spans="1:5">
+    <row r="272" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>275</v>
       </c>
@@ -4979,12 +5067,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="273" spans="1:5">
+    <row r="273" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="274" spans="1:5">
+    <row r="274" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>277</v>
       </c>
@@ -5001,12 +5089,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="275" spans="1:5">
+    <row r="275" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A275" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="276" spans="1:5">
+    <row r="276" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A276" t="s">
         <v>279</v>
       </c>
@@ -5023,12 +5111,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="277" spans="1:5">
+    <row r="277" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A277" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="278" spans="1:5">
+    <row r="278" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A278" t="s">
         <v>281</v>
       </c>
@@ -5045,12 +5133,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="279" spans="1:5">
+    <row r="279" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A279" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="280" spans="1:5">
+    <row r="280" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
         <v>283</v>
       </c>
@@ -5067,52 +5155,52 @@
         <v>200</v>
       </c>
     </row>
-    <row r="281" spans="1:5">
+    <row r="281" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
         <v>284</v>
       </c>
     </row>
-    <row r="282" spans="1:5">
+    <row r="282" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="283" spans="1:5">
+    <row r="283" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="284" spans="1:5">
+    <row r="284" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="285" spans="1:5">
+    <row r="285" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="286" spans="1:5">
+    <row r="286" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="287" spans="1:5">
+    <row r="287" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="288" spans="1:5">
+    <row r="288" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="289" spans="1:5">
+    <row r="289" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="290" spans="1:5">
+    <row r="290" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>293</v>
       </c>
@@ -5129,12 +5217,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="291" spans="1:5">
+    <row r="291" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="292" spans="1:5">
+    <row r="292" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>295</v>
       </c>
@@ -5151,12 +5239,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="293" spans="1:5">
+    <row r="293" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="294" spans="1:5">
+    <row r="294" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>297</v>
       </c>
@@ -5173,12 +5261,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="295" spans="1:5">
+    <row r="295" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="296" spans="1:5">
+    <row r="296" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>299</v>
       </c>
@@ -5195,12 +5283,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="297" spans="1:5">
+    <row r="297" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="298" spans="1:5">
+    <row r="298" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>301</v>
       </c>
@@ -5217,12 +5305,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="299" spans="1:5">
+    <row r="299" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="300" spans="1:5">
+    <row r="300" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
         <v>303</v>
       </c>
@@ -5239,12 +5327,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="301" spans="1:5">
+    <row r="301" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="302" spans="1:5">
+    <row r="302" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
         <v>305</v>
       </c>
@@ -5261,12 +5349,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="303" spans="1:5">
+    <row r="303" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="304" spans="1:5">
+    <row r="304" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
         <v>307</v>
       </c>
@@ -5283,52 +5371,52 @@
         <v>200</v>
       </c>
     </row>
-    <row r="305" spans="1:5">
+    <row r="305" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A305" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="306" spans="1:5">
+    <row r="306" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="307" spans="1:5">
+    <row r="307" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A307" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="308" spans="1:5">
+    <row r="308" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A308" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="309" spans="1:5">
+    <row r="309" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A309" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="310" spans="1:5">
+    <row r="310" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A310" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="311" spans="1:5">
+    <row r="311" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A311" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="312" spans="1:5">
+    <row r="312" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A312" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="313" spans="1:5">
+    <row r="313" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A313" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="314" spans="1:5">
+    <row r="314" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A314" t="s">
         <v>317</v>
       </c>
@@ -5345,12 +5433,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="315" spans="1:5">
+    <row r="315" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A315" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="316" spans="1:5">
+    <row r="316" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A316" t="s">
         <v>319</v>
       </c>
@@ -5367,12 +5455,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="317" spans="1:5">
+    <row r="317" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A317" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="318" spans="1:5">
+    <row r="318" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A318" t="s">
         <v>321</v>
       </c>
@@ -5389,12 +5477,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="319" spans="1:5">
+    <row r="319" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A319" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="320" spans="1:5">
+    <row r="320" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A320" t="s">
         <v>323</v>
       </c>
@@ -5411,12 +5499,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="321" spans="1:5">
+    <row r="321" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A321" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="322" spans="1:5">
+    <row r="322" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A322" t="s">
         <v>325</v>
       </c>
@@ -5433,12 +5521,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="323" spans="1:5">
+    <row r="323" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A323" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="324" spans="1:5">
+    <row r="324" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A324" t="s">
         <v>327</v>
       </c>
@@ -5455,12 +5543,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="325" spans="1:5">
+    <row r="325" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A325" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="326" spans="1:5">
+    <row r="326" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A326" t="s">
         <v>329</v>
       </c>
@@ -5477,12 +5565,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="327" spans="1:5">
+    <row r="327" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A327" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="328" spans="1:5">
+    <row r="328" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A328" t="s">
         <v>331</v>
       </c>
@@ -5499,52 +5587,52 @@
         <v>200</v>
       </c>
     </row>
-    <row r="329" spans="1:5">
+    <row r="329" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A329" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="330" spans="1:5">
+    <row r="330" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A330" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="331" spans="1:5">
+    <row r="331" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A331" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="332" spans="1:5">
+    <row r="332" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A332" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="333" spans="1:5">
+    <row r="333" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A333" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="334" spans="1:5">
+    <row r="334" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A334" t="s">
         <v>337</v>
       </c>
     </row>
-    <row r="335" spans="1:5">
+    <row r="335" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A335" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="336" spans="1:5">
+    <row r="336" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A336" t="s">
         <v>339</v>
       </c>
     </row>
-    <row r="337" spans="1:5">
+    <row r="337" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A337" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="338" spans="1:5">
+    <row r="338" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A338" t="s">
         <v>341</v>
       </c>
@@ -5561,12 +5649,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="339" spans="1:5">
+    <row r="339" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A339" t="s">
         <v>342</v>
       </c>
     </row>
-    <row r="340" spans="1:5">
+    <row r="340" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A340" t="s">
         <v>343</v>
       </c>
@@ -5583,12 +5671,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="341" spans="1:5">
+    <row r="341" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A341" t="s">
         <v>344</v>
       </c>
     </row>
-    <row r="342" spans="1:5">
+    <row r="342" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A342" t="s">
         <v>345</v>
       </c>
@@ -5605,12 +5693,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="343" spans="1:5">
+    <row r="343" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A343" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="344" spans="1:5">
+    <row r="344" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A344" t="s">
         <v>347</v>
       </c>
@@ -5627,12 +5715,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="345" spans="1:5">
+    <row r="345" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A345" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="346" spans="1:5">
+    <row r="346" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A346" t="s">
         <v>349</v>
       </c>
@@ -5649,12 +5737,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="347" spans="1:5">
+    <row r="347" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A347" t="s">
         <v>350</v>
       </c>
     </row>
-    <row r="348" spans="1:5">
+    <row r="348" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A348" t="s">
         <v>351</v>
       </c>
@@ -5671,12 +5759,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="349" spans="1:5">
+    <row r="349" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A349" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="350" spans="1:5">
+    <row r="350" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A350" t="s">
         <v>353</v>
       </c>
@@ -5693,12 +5781,12 @@
         <v>200</v>
       </c>
     </row>
-    <row r="351" spans="1:5">
+    <row r="351" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A351" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="352" spans="1:5">
+    <row r="352" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A352" t="s">
         <v>355</v>
       </c>
@@ -5715,167 +5803,167 @@
         <v>200</v>
       </c>
     </row>
-    <row r="353" spans="1:1">
+    <row r="353" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A353" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="354" spans="1:1">
+    <row r="354" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A354" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="355" spans="1:1">
+    <row r="355" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A355" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="356" spans="1:1">
+    <row r="356" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A356" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="357" spans="1:1">
+    <row r="357" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A357" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="358" spans="1:1">
+    <row r="358" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A358" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="359" spans="1:1">
+    <row r="359" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A359" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="360" spans="1:1">
+    <row r="360" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A360" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="361" spans="1:1">
+    <row r="361" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A361" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="362" spans="1:1">
+    <row r="362" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A362" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="363" spans="1:1">
+    <row r="363" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A363" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="364" spans="1:1">
+    <row r="364" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A364" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="365" spans="1:1">
+    <row r="365" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A365" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="366" spans="1:1">
+    <row r="366" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A366" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="367" spans="1:1">
+    <row r="367" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A367" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="368" spans="1:1">
+    <row r="368" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A368" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="369" spans="1:1">
+    <row r="369" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A369" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="370" spans="1:1">
+    <row r="370" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A370" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="371" spans="1:1">
+    <row r="371" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A371" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="372" spans="1:1">
+    <row r="372" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A372" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="373" spans="1:1">
+    <row r="373" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A373" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="374" spans="1:1">
+    <row r="374" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A374" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="375" spans="1:1">
+    <row r="375" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A375" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="376" spans="1:1">
+    <row r="376" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A376" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="377" spans="1:1">
+    <row r="377" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A377" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="378" spans="1:1">
+    <row r="378" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A378" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="379" spans="1:1">
+    <row r="379" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A379" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="380" spans="1:1">
+    <row r="380" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A380" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="381" spans="1:1">
+    <row r="381" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A381" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="382" spans="1:1">
+    <row r="382" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A382" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="383" spans="1:1">
+    <row r="383" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A383" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="384" spans="1:1">
+    <row r="384" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A384" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="385" spans="1:1">
+    <row r="385" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A385" t="s">
         <v>388</v>
       </c>
@@ -5886,27 +5974,27 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Y17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="53.7109375" customWidth="1"/>
-    <col min="2" max="3" width="54.7109375" customWidth="1"/>
-    <col min="4" max="4" width="45.7109375" customWidth="1"/>
-    <col min="5" max="6" width="41.7109375" customWidth="1"/>
-    <col min="7" max="8" width="45.7109375" customWidth="1"/>
-    <col min="9" max="9" width="41.7109375" customWidth="1"/>
-    <col min="10" max="10" width="37.7109375" customWidth="1"/>
-    <col min="11" max="11" width="41.7109375" customWidth="1"/>
-    <col min="12" max="12" width="37.7109375" customWidth="1"/>
-    <col min="13" max="13" width="41.7109375" customWidth="1"/>
-    <col min="14" max="14" width="37.7109375" customWidth="1"/>
-    <col min="15" max="15" width="41.7109375" customWidth="1"/>
-    <col min="16" max="16" width="37.7109375" customWidth="1"/>
-    <col min="17" max="24" width="5.7109375" customWidth="1"/>
+    <col min="1" max="1" width="53.6640625" customWidth="1"/>
+    <col min="2" max="3" width="54.6640625" customWidth="1"/>
+    <col min="4" max="4" width="45.6640625" customWidth="1"/>
+    <col min="5" max="6" width="41.6640625" customWidth="1"/>
+    <col min="7" max="8" width="45.6640625" customWidth="1"/>
+    <col min="9" max="9" width="41.6640625" customWidth="1"/>
+    <col min="10" max="10" width="37.6640625" customWidth="1"/>
+    <col min="11" max="11" width="41.6640625" customWidth="1"/>
+    <col min="12" max="12" width="37.6640625" customWidth="1"/>
+    <col min="13" max="13" width="41.6640625" customWidth="1"/>
+    <col min="14" max="14" width="37.6640625" customWidth="1"/>
+    <col min="15" max="15" width="41.6640625" customWidth="1"/>
+    <col min="16" max="16" width="37.6640625" customWidth="1"/>
+    <col min="17" max="24" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>733</v>
       </c>
@@ -5983,7 +6071,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="2" spans="1:25" s="2" customFormat="1">
+    <row r="2" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>734</v>
       </c>
@@ -6000,7 +6088,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>735</v>
       </c>
@@ -6029,7 +6117,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="1:25" s="2" customFormat="1">
+    <row r="4" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>736</v>
       </c>
@@ -6058,7 +6146,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>737</v>
       </c>
@@ -6087,7 +6175,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="6" spans="1:25" s="2" customFormat="1">
+    <row r="6" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>738</v>
       </c>
@@ -6098,7 +6186,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>739</v>
       </c>
@@ -6151,7 +6239,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="8" spans="1:25" s="2" customFormat="1">
+    <row r="8" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>740</v>
       </c>
@@ -6201,7 +6289,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="9" spans="1:25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>741</v>
       </c>
@@ -6218,7 +6306,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="10" spans="1:25" s="2" customFormat="1">
+    <row r="10" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>742</v>
       </c>
@@ -6235,7 +6323,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="11" spans="1:25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>743</v>
       </c>
@@ -6243,13 +6331,22 @@
         <v>458</v>
       </c>
       <c r="C11" t="s">
-        <v>459</v>
+        <v>753</v>
       </c>
       <c r="D11" t="s">
         <v>460</v>
       </c>
-    </row>
-    <row r="12" spans="1:25" s="2" customFormat="1">
+      <c r="E11" t="s">
+        <v>753</v>
+      </c>
+      <c r="G11" t="s">
+        <v>459</v>
+      </c>
+      <c r="H11" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>744</v>
       </c>
@@ -6266,7 +6363,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>745</v>
       </c>
@@ -6295,7 +6392,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="14" spans="1:25" s="2" customFormat="1">
+    <row r="14" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>746</v>
       </c>
@@ -6324,7 +6421,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="15" spans="1:25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>747</v>
       </c>
@@ -6353,7 +6450,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="16" spans="1:25" s="2" customFormat="1">
+    <row r="16" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>748</v>
       </c>
@@ -6382,7 +6479,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>749</v>
       </c>
@@ -6393,14 +6490,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Y17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="24" width="5.7109375" customWidth="1"/>
+    <col min="1" max="24" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>733</v>
       </c>
@@ -6477,7 +6574,7 @@
         <v>732</v>
       </c>
     </row>
-    <row r="2" spans="1:25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>734</v>
       </c>
@@ -6494,7 +6591,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>735</v>
       </c>
@@ -6523,7 +6620,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="4" spans="1:25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>736</v>
       </c>
@@ -6552,7 +6649,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>737</v>
       </c>
@@ -6581,7 +6678,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="6" spans="1:25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>738</v>
       </c>
@@ -6592,7 +6689,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>739</v>
       </c>
@@ -6645,7 +6742,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="8" spans="1:25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>740</v>
       </c>
@@ -6695,7 +6792,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="9" spans="1:25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>741</v>
       </c>
@@ -6712,7 +6809,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>742</v>
       </c>
@@ -6729,21 +6826,30 @@
         <v>736</v>
       </c>
     </row>
-    <row r="11" spans="1:25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>743</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>736</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>736</v>
+      <c r="C11" s="6" t="s">
+        <v>755</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>736</v>
       </c>
-    </row>
-    <row r="12" spans="1:25">
+      <c r="E11" s="6" t="s">
+        <v>755</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>736</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>744</v>
       </c>
@@ -6760,7 +6866,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>745</v>
       </c>
@@ -6789,7 +6895,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="14" spans="1:25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>746</v>
       </c>
@@ -6818,7 +6924,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="15" spans="1:25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>747</v>
       </c>
@@ -6847,7 +6953,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="16" spans="1:25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>748</v>
       </c>
@@ -6876,7 +6982,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>749</v>
       </c>

</xml_diff>